<commit_message>
metrics to trends init
</commit_message>
<xml_diff>
--- a/mark59-datahunter-samples/mark59serverprofiles.xlsx
+++ b/mark59-datahunter-samples/mark59serverprofiles.xlsx
@@ -81,7 +81,7 @@
     <t>DemoLINUX-DataHunterSeleniumRunCheck</t>
   </si>
   <si>
-    <t>Loads Trend Analysis (H2 database).  See:&lt;br&gt;http://localhost:8083/metrics/trending?reqApp=DataHunter</t>
+    <t>Loads Trend Analysis (H2 database).  See:&lt;br&gt;http://localhost:8083/mark59-trends/trending?reqApp=DataHunter</t>
   </si>
   <si>
     <t>DemoWIN-DataHunterSeleniumDeployAndExecute</t>
@@ -220,23 +220,23 @@
  echo Running Directly From Server Metrics Web (cmd DataHunterSeleniumDeployAndExecute) &amp; 
  echo  SERVER_METRICS_WEB_BASE_DIR: %SERVER_METRICS_WEB_BASE_DIR% &amp; 
  cd /D %SERVER_METRICS_WEB_BASE_DIR% &amp;  
- cd ..\dataHunterPerformanceTestSamples &amp; 
+ cd ..\mark59-datahunter-samples &amp; 
  DEL C:\apache-jmeter\bin\mark59.properties &amp; COPY .\mark59.properties C:\apache-jmeter\bin &amp;
  DEL C:\apache-jmeter\bin\chromedriver.exe  &amp; COPY .\chromedriver.exe  C:\apache-jmeter\bin &amp;
- DEL C:\apache-jmeter\lib\ext\mark59-server-metrics.jar &amp;
- COPY ..\mark59-server-metrics\target\mark59-server-metrics.jar  C:\apache-jmeter\lib\ext &amp; 
- DEL C:\apache-jmeter\lib\ext\dataHunterPerformanceTestSamples.jar &amp; 
- COPY .\target\dataHunterPerformanceTestSamples.jar  C:\apache-jmeter\lib\ext &amp;
- RMDIR /S /Q C:\apache-jmeter\lib\ext\dataHunterPerformanceTestSamples-dependencies &amp;
- MKDIR C:\apache-jmeter\lib\ext\dataHunterPerformanceTestSamples-dependencies &amp;
- COPY .\target\dataHunterPerformanceTestSamples-dependencies  C:\apache-jmeter\lib\ext\dataHunterPerformanceTestSamples-dependencies &amp;
+ DEL C:\apache-jmeter\lib\ext\mark59-metrics.jar &amp;
+ COPY ..\mark59-metrics\target\mark59-metrics.jar  C:\apache-jmeter\lib\ext &amp; 
+ DEL C:\apache-jmeter\lib\ext\mark59-datahunter-samples.jar &amp; 
+ COPY .\target\mark59-datahunter-samples.jar  C:\apache-jmeter\lib\ext &amp;
+ RMDIR /S /Q C:\apache-jmeter\lib\ext\mark59-datahunter-samples-dependencies &amp;
+ MKDIR C:\apache-jmeter\lib\ext\mark59-datahunter-samples-dependencies &amp;
+ COPY .\target\mark59-datahunter-samples-dependencies  C:\apache-jmeter\lib\ext\mark59-datahunter-samples-dependencies &amp;
  mkdir C:\Mark59_Runs &amp;
  mkdir C:\Mark59_Runs\Jmeter_Results &amp;
  mkdir C:\Mark59_Runs\Jmeter_Results\DataHunter &amp;
  set path=%path%;C:\Windows\System32;C:\windows\system32\wbem &amp; 
  cd /D C:\apache-jmeter\bin &amp;
  echo Starting JMeter DataHunter test ... &amp;  
- jmeter -n -X -f -t %SERVER_METRICS_WEB_BASE_DIR%\..\dataHunterPerformanceTestSamples\test-plans\DataHunterSeleniumTestPlan.jmx -l C:\Mark59_Runs\Jmeter_Results\DataHunter\DataHunterTestResults.csv -JForceTxnFailPercent=0 -JDataHunterUrl=http://localhost:8081/dataHunter -JStartCdpListeners=false &amp;
+ jmeter -n -X -f -t %SERVER_METRICS_WEB_BASE_DIR%\..\mark59-datahunter-samples\test-plans\DataHunterSeleniumTestPlan.jmx -l C:\Mark59_Runs\Jmeter_Results\DataHunter\DataHunterTestResults.csv -JForceTxnFailPercent=0 -JDataHunterUrl=http://localhost:8081/mark59-datahunter -JStartCdpListeners=false &amp;
  PAUSE
 '
 </t>
@@ -245,7 +245,7 @@
     <t>N</t>
   </si>
   <si>
-    <t xml:space="preserve">refer DeployDataHunterTestArtifactsToJmeter.bat and DataHunterExecuteJmeterTest.bat in dataHunterPerformanceTestSamples </t>
+    <t xml:space="preserve">refer DeployDataHunterTestArtifactsToJmeter.bat and DataHunterExecuteJmeterTest.bat in mark59-datahunter-samples </t>
   </si>
   <si>
     <t>[]</t>
@@ -254,16 +254,16 @@
     <t>echo This script runs the JMeter deploy in the background, then opens a terminal for JMeter execution.
 echo starting from $PWD;
 {   # try  
-    cd ../dataHunterPerformanceTestSamples &amp;&amp; 
+    cd ../mark59-datahunter-samples &amp;&amp; 
     DH_TEST_SAMPLES_DIR=$(pwd) &amp;&amp; 
-    echo dataHunterPerformanceTestSamples base dir is $DH_TEST_SAMPLES_DIR &amp;&amp;
+    echo mark59-datahunter-samples base dir is $DH_TEST_SAMPLES_DIR &amp;&amp;
     cp ./mark59.properties ~/apache-jmeter/bin/mark59.properties &amp;&amp;
     cp ./chromedriver ~/apache-jmeter/bin/chromedriver &amp;&amp; 
-    cp ../mark59-server-metrics/target/mark59-server-metrics.jar  ~/apache-jmeter/lib/ext/mark59-server-metrics.jar &amp;&amp; 
-    cp ./target/dataHunterPerformanceTestSamples.jar  ~/apache-jmeter/lib/ext/dataHunterPerformanceTestSamples.jar &amp;&amp; 
+    cp ../mark59-metrics/target/mark59-metrics.jar  ~/apache-jmeter/lib/ext/mark59-metrics.jar &amp;&amp; 
+    cp ./target/mark59-datahunter-samples.jar  ~/apache-jmeter/lib/ext/mark59-datahunter-samples.jar &amp;&amp; 
     mkdir -p ~/Mark59_Runs/Jmeter_Results/DataHunter &amp;&amp;
-    rm -rf ~/apache-jmeter/lib/ext/dataHunterPerformanceTestSamples-dependencies &amp;&amp;
-    cp -r ./target/dataHunterPerformanceTestSamples-dependencies ~/apache-jmeter/lib/ext/dataHunterPerformanceTestSamples-dependencies &amp;&amp;
+    rm -rf ~/apache-jmeter/lib/ext/mark59-datahunter-samples-dependencies &amp;&amp;
+    cp -r ./target/mark59-datahunter-samples-dependencies ~/apache-jmeter/lib/ext/mark59-datahunter-samples-dependencies &amp;&amp;
     gnome-terminal -- sh -c "~/apache-jmeter/bin/jmeter -n -X -f -t $DH_TEST_SAMPLES_DIR/test-plans/DataHunterSeleniumTestPlan.jmx -l ~/Mark59_Runs/Jmeter_Results/DataHunter/DataHunterTestResults.csv -JForceTxnFailPercent=0 -JStartCdpListeners=false; exec bash"
 } || { # catch 
     echo Deploy was unsuccessful! 
@@ -298,22 +298,22 @@
   </si>
   <si>
     <t xml:space="preserve">process call create 'cmd.exe /c 
- echo Load DataHunter Test Results into  Mark59 Metrics (Trend Analysis) h2 database. &amp; 
+ echo Load DataHunter Test Results into  Mark59 Trends Analysis h2 database. &amp; 
  cd /D  %SERVER_METRICS_WEB_BASE_DIR% &amp; 
- cd ../metricsRuncheck &amp;  
- java -jar ./target/metricsRuncheck.jar -a DataHunter -i C:\Mark59_Runs\Jmeter_Results\DataHunter -d h2 &amp;
+ cd ../mark59-trends-load &amp;  
+ java -jar ./target/mark59-trends-load.jar -a DataHunter -i C:\Mark59_Runs\Jmeter_Results\DataHunter -d h2 &amp;
  PAUSE
 '
 </t>
   </si>
   <si>
-    <t xml:space="preserve">echo This script runs metricsRuncheck,to load results from a DataHunter test run into the Metrics Trend Analysis Graph.
+    <t xml:space="preserve">echo This script runs mark59-trends-load,to load results from a DataHunter test run into the Metrics Trend Analysis Graph.
 echo starting from $PWD;
 {   # try  
-    cd ../metricsRuncheck/target &amp;&amp;
-    gnome-terminal -- sh -c "java -jar metricsRuncheck.jar -a DataHunter -i ~/Mark59_Runs/Jmeter_Results/DataHunter -d h2; exec bash"
+    cd ../mark59-trends-load/target &amp;&amp;
+    gnome-terminal -- sh -c "java -jar mark59-trends-load.jar -a DataHunter -i ~/Mark59_Runs/Jmeter_Results/DataHunter -d h2; exec bash"
 } || { # catch 
-    echo attempt to execute metricsRuncheck has failed! 
+    echo attempt to execute mark59-trends-load has failed! 
 }
 </t>
   </si>
@@ -802,7 +802,7 @@
     <col min="7" max="7" width="19.46484375" customWidth="true" bestFit="true"/>
     <col min="8" max="8" width="19.5390625" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="23.23828125" customWidth="true" bestFit="true"/>
-    <col min="10" max="10" width="102.359375" customWidth="true" bestFit="true"/>
+    <col min="10" max="10" width="103.01953125" customWidth="true" bestFit="true"/>
     <col min="11" max="11" width="71.546875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
@@ -1523,7 +1523,7 @@
     <col min="2" max="2" width="17.41015625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="255.0" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="16.45703125" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="117.37890625" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="109.81640625" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="62.10546875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>

</xml_diff>